<commit_message>
Pipeline listo para el entrenamiento final
</commit_message>
<xml_diff>
--- a/resultados/Resultados_FacebookAI_roberta-base.xlsx
+++ b/resultados/Resultados_FacebookAI_roberta-base.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UMA\TFG\TFG-Sistema-Recomendacion-Personalidad\resultados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1331E8-6377-4BF3-82B4-37B48BFD3284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F73A397-7FA5-48DB-A23F-163C1E45DE9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -528,6 +528,22 @@
  [217 307]]</t>
   </si>
   <si>
+    <t>0: 0.37
+1: 0.89</t>
+  </si>
+  <si>
+    <t>0: 0.42
+1: 0.88</t>
+  </si>
+  <si>
+    <t>0: 0.23
+1: 0.95</t>
+  </si>
+  <si>
+    <t>0: 0.29
+1: 0.92</t>
+  </si>
+  <si>
     <t>0: 0.46
 1: 0.89</t>
   </si>
@@ -620,10 +636,6 @@
 1: 0.90</t>
   </si>
   <si>
-    <t>0: 0.37
-1: 0.89</t>
-  </si>
-  <si>
     <t>[[47 73]
  [87 661]]</t>
   </si>
@@ -726,18 +738,6 @@
   <si>
     <t>[[87 113]
  [87 581]]</t>
-  </si>
-  <si>
-    <t>0: 0.42
-1: 0.88</t>
-  </si>
-  <si>
-    <t>0: 0.23
-1: 0.95</t>
-  </si>
-  <si>
-    <t>0: 0.29
-1: 0.92</t>
   </si>
   <si>
     <t>[[27 93]
@@ -2422,13 +2422,13 @@
         <v>7</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>11</v>
@@ -2437,7 +2437,7 @@
         <v>0.74</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -2464,7 +2464,7 @@
         <v>0.75</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -2547,13 +2547,13 @@
         <v>33</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>11</v>
@@ -2562,7 +2562,7 @@
         <v>0.76</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -2574,7 +2574,7 @@
         <v>38</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>40</v>
@@ -2589,7 +2589,7 @@
         <v>0.85</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
@@ -2672,13 +2672,13 @@
         <v>53</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>11</v>
@@ -2687,7 +2687,7 @@
         <v>0.76</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -2699,13 +2699,13 @@
         <v>58</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>17</v>
@@ -2714,7 +2714,7 @@
         <v>0.77</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -2797,13 +2797,13 @@
         <v>74</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>77</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="E17" s="12" t="s">
         <v>11</v>
@@ -2812,7 +2812,7 @@
         <v>0.72</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
@@ -2824,13 +2824,13 @@
         <v>79</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C18" s="12" t="s">
         <v>39</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>158</v>
+        <v>135</v>
       </c>
       <c r="E18" s="12" t="s">
         <v>17</v>
@@ -2839,7 +2839,7 @@
         <v>0.82</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
@@ -2922,13 +2922,13 @@
         <v>95</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E22" s="25" t="s">
         <v>11</v>
@@ -2937,7 +2937,7 @@
         <v>0.48</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
@@ -2952,10 +2952,10 @@
         <v>101</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="E23" s="25" t="s">
         <v>17</v>
@@ -2964,7 +2964,7 @@
         <v>0.49</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
@@ -3047,13 +3047,13 @@
         <v>114</v>
       </c>
       <c r="B27" s="28" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="E27" s="28" t="s">
         <v>11</v>
@@ -3062,7 +3062,7 @@
         <v>0.62</v>
       </c>
       <c r="G27" s="29" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
@@ -3074,13 +3074,13 @@
         <v>119</v>
       </c>
       <c r="B28" s="28" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C28" s="28" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E28" s="28" t="s">
         <v>17</v>
@@ -3089,7 +3089,7 @@
         <v>0.68</v>
       </c>
       <c r="G28" s="29" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
@@ -3205,10 +3205,10 @@
         <v>8</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>11</v>
@@ -3217,7 +3217,7 @@
         <v>0.73</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -3229,10 +3229,10 @@
         <v>13</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>50</v>
@@ -3244,7 +3244,7 @@
         <v>0.72</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -3327,13 +3327,13 @@
         <v>33</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>11</v>
@@ -3342,7 +3342,7 @@
         <v>0.77</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -3354,13 +3354,13 @@
         <v>38</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>185</v>
+        <v>136</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>186</v>
+        <v>137</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>187</v>
+        <v>138</v>
       </c>
       <c r="E8" s="8" t="s">
         <v>17</v>
@@ -3950,8 +3950,8 @@
     <col min="8" max="9" width="9.140625" style="1" customWidth="1"/>
     <col min="10" max="10" width="13.42578125" style="1" customWidth="1"/>
     <col min="11" max="11" width="45.85546875" style="1" customWidth="1"/>
-    <col min="12" max="13" width="9.140625" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="1"/>
+    <col min="12" max="14" width="9.140625" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Resultados y modelos de la nueva version + Roberta Finetunned
</commit_message>
<xml_diff>
--- a/resultados/Resultados_FacebookAI_roberta-base.xlsx
+++ b/resultados/Resultados_FacebookAI_roberta-base.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UMA\TFG\TFG-Sistema-Recomendacion-Personalidad\resultados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F73A397-7FA5-48DB-A23F-163C1E45DE9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF547AF1-D74B-4DF4-89AD-A6B2E84E20A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="302">
   <si>
     <t>Modelos</t>
   </si>
@@ -45,9 +45,6 @@
   </si>
   <si>
     <t>Matriz Confusion</t>
-  </si>
-  <si>
-    <t>Regresión Logística E/I</t>
   </si>
   <si>
     <t>0: 0.45
@@ -58,29 +55,14 @@
 1: 0.77</t>
   </si>
   <si>
-    <t>0: 0.53
-1: 0.82</t>
-  </si>
-  <si>
     <t>0: 200
 1: 668</t>
   </si>
   <si>
-    <t>[[129 71]
- [155 513]]</t>
-  </si>
-  <si>
-    <t>Regresión Logística S/N</t>
-  </si>
-  <si>
     <t>0: 0.24
 1: 0.90</t>
   </si>
   <si>
-    <t>0: 0.47
-1: 0.77</t>
-  </si>
-  <si>
     <t>0: 0.32
 1: 0.83</t>
   </si>
@@ -89,17 +71,10 @@
 1: 748</t>
   </si>
   <si>
-    <t>[[56 64]
- [175 573]]</t>
-  </si>
-  <si>
     <t>Parametros</t>
   </si>
   <si>
     <t>{'penalty': None, 'C': 9.732719859279047, 'solver': 'lbfgs', 'tol': 0.00010564097578389837, 'class_weight': 'balanced', 'random_state': 42, 'n_jobs': -1, 'max_iter': 5000}</t>
-  </si>
-  <si>
-    <t>Regresión Logística T/F</t>
   </si>
   <si>
     <t>0: 0.71
@@ -118,111 +93,25 @@
 1: 470</t>
   </si>
   <si>
-    <t>[[318 80]
- [131 339]]</t>
-  </si>
-  <si>
-    <t>Regresión Logística J/P</t>
-  </si>
-  <si>
-    <t>0: 0.51
-1: 0.70</t>
-  </si>
-  <si>
-    <t>0: 0.58
-1: 0.64</t>
-  </si>
-  <si>
-    <t>0: 0.54
-1: 0.67</t>
-  </si>
-  <si>
     <t>0: 344
 1: 524</t>
   </si>
   <si>
-    <t>[[198 146]
- [190 334]]</t>
-  </si>
-  <si>
-    <t>XGBoost E/I</t>
-  </si>
-  <si>
     <t>0: 0.51
 1: 0.83</t>
   </si>
   <si>
     <t>0: 0.39
-1: 0.89</t>
-  </si>
-  <si>
-    <t>0: 0.44
-1: 0.86</t>
-  </si>
-  <si>
-    <t>[[78 122]
- [76 592]]</t>
-  </si>
-  <si>
-    <t>XGBoost S/N</t>
-  </si>
-  <si>
-    <t>0: 0.39
 1: 0.88</t>
   </si>
   <si>
-    <t>0: 0.22
-1: 0.95</t>
-  </si>
-  <si>
-    <t>0: 0.28
-1: 0.91</t>
-  </si>
-  <si>
-    <t>[[26 94]
- [41 707]]</t>
-  </si>
-  <si>
     <t>{'n_estimators': 352, 'max_depth': 8, 'learning_rate': 0.041694500859353036, 'subsample': 0.6688508428769014, 'colsample_bytree': 0.6246885857257476, 'gamma': 0.6844100651211652, 'tree_method': 'hist', 'device': 'cuda', 'random_state': 42, 'n_jobs': 1}</t>
-  </si>
-  <si>
-    <t>XGBoost T/F</t>
-  </si>
-  <si>
-    <t>0: 0.76
-1: 0.79</t>
-  </si>
-  <si>
-    <t>0: 0.75
-1: 0.80</t>
-  </si>
-  <si>
-    <t>[[297 101]
- [93 377]]</t>
-  </si>
-  <si>
-    <t>XGBoost J/P</t>
   </si>
   <si>
     <t>0: 0.56
 1: 0.65</t>
   </si>
   <si>
-    <t>0: 0.33
-1: 0.83</t>
-  </si>
-  <si>
-    <t>0: 0.42
-1: 0.73</t>
-  </si>
-  <si>
-    <t>[[114 230]
- [88 436]]</t>
-  </si>
-  <si>
-    <t>LinearSVM E/I</t>
-  </si>
-  <si>
     <t>0: 0.44
 1: 0.90</t>
   </si>
@@ -239,48 +128,15 @@
  [184 484]]</t>
   </si>
   <si>
-    <t>LinearSVM S/N</t>
-  </si>
-  <si>
     <t>0: 0.27
 1: 0.91</t>
   </si>
   <si>
-    <t>0: 0.50
-1: 0.78</t>
-  </si>
-  <si>
     <t>0: 0.35
 1: 0.84</t>
   </si>
   <si>
-    <t>[[60 60]
- [162 586]]</t>
-  </si>
-  <si>
     <t>{'loss': 'squared_hinge', 'C': 9.605448156429867, 'tol': 0.0004119653918147926, 'fit_intercept': False, 'random_state': 42, 'class_weight': 'balanced', 'max_iter': 5000}</t>
-  </si>
-  <si>
-    <t>LinearSVM T/F</t>
-  </si>
-  <si>
-    <t>0: 0.72
-1: 0.82</t>
-  </si>
-  <si>
-    <t>0: 0.80
-1: 0.74</t>
-  </si>
-  <si>
-    <t>0: 0.76
-1: 0.78</t>
-  </si>
-  <si>
-    <t>[[319 79]
- [121 349]]</t>
-  </si>
-  <si>
-    <t>LinearSVM J/P</t>
   </si>
   <si>
     <t>0: 0.47
@@ -299,9 +155,6 @@
  [289 235]]</t>
   </si>
   <si>
-    <t>MLP E/I</t>
-  </si>
-  <si>
     <t>0: 0.41
 1: 0.87</t>
   </si>
@@ -318,13 +171,6 @@
  [187 481]]</t>
   </si>
   <si>
-    <t>MLP S/N</t>
-  </si>
-  <si>
-    <t>0: 0.37
-1: 0.90</t>
-  </si>
-  <si>
     <t>0: 0.38
 1: 0.89</t>
   </si>
@@ -333,14 +179,7 @@
 1: 0.90</t>
   </si>
   <si>
-    <t>[[46 74]
- [79 669]]</t>
-  </si>
-  <si>
     <t>{'hidden_layer_sizes': (256, 128, 64), 'activation': 'tanh', 'solver': 'adam', 'learning_rate': 'constant', 'learning_rate_init': 0.001, 'early_stopping': True, 'max_iter': 6000, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>MLP T/F</t>
   </si>
   <si>
     <t>0: 0.72
@@ -359,9 +198,6 @@
  [126 344]]</t>
   </si>
   <si>
-    <t>MLP J/P</t>
-  </si>
-  <si>
     <t>0: 0.62
 1: 0.68</t>
   </si>
@@ -378,9 +214,6 @@
  [79 445]]</t>
   </si>
   <si>
-    <t>KNeighboursClassifier E/I</t>
-  </si>
-  <si>
     <t>0: 0.27
 1: 0.84</t>
   </si>
@@ -397,9 +230,6 @@
  [403 265]]</t>
   </si>
   <si>
-    <t>KNeighboursClassifier S/N</t>
-  </si>
-  <si>
     <t>0: 0.15
 1: 0.88</t>
   </si>
@@ -419,9 +249,6 @@
     <t>{'n_neighbors': 2, 'weights': 'distance', 'algorithm': 'brute', 'leaf_size': 14, 'metric': 'cosine', 'n_jobs': -1}</t>
   </si>
   <si>
-    <t>KNeighboursClassifier T/F</t>
-  </si>
-  <si>
     <t>0: 0.57
 1: 0.64</t>
   </si>
@@ -430,9 +257,6 @@
  [168 302]]</t>
   </si>
   <si>
-    <t>KNeighboursClassifier J/P</t>
-  </si>
-  <si>
     <t>0: 0.44
 1: 0.63</t>
   </si>
@@ -449,9 +273,6 @@
  [174 350]]</t>
   </si>
   <si>
-    <t>DecisionTreeClassifier E/I</t>
-  </si>
-  <si>
     <t>0: 0.29
 1: 0.81</t>
   </si>
@@ -468,9 +289,6 @@
  [245 423]]</t>
   </si>
   <si>
-    <t>DecisionTreeClassifier S/N</t>
-  </si>
-  <si>
     <t>0: 0.15
 1: 0.86</t>
   </si>
@@ -490,9 +308,6 @@
     <t>{'criterion': 'gini', 'max_depth': 15, 'min_samples_split': 9, 'min_samples_leaf': 4, 'max_features': None, 'class_weight': None, 'random_state': 42}</t>
   </si>
   <si>
-    <t>DecisionTreeClassifier T/F</t>
-  </si>
-  <si>
     <t>0: 0.59
 1: 0.67</t>
   </si>
@@ -509,9 +324,6 @@
  [179 291]]</t>
   </si>
   <si>
-    <t>DecisionTreeClassifier J/P</t>
-  </si>
-  <si>
     <t>0: 0.43
 1: 0.63</t>
   </si>
@@ -528,10 +340,76 @@
  [217 307]]</t>
   </si>
   <si>
+    <t>LR E/I</t>
+  </si>
+  <si>
+    <t>0: 0.46
+1: 0.88</t>
+  </si>
+  <si>
+    <t>0: 0.54
+1: 0.82</t>
+  </si>
+  <si>
+    <t>[[129 71]
+ [153 515]]</t>
+  </si>
+  <si>
+    <t>LR S/N</t>
+  </si>
+  <si>
+    <t>0: 0.47
+1: 0.76</t>
+  </si>
+  <si>
+    <t>[[56 64]
+ [176 572]]</t>
+  </si>
+  <si>
+    <t>LR T/F</t>
+  </si>
+  <si>
+    <t>[[319 79]
+ [131 339]]</t>
+  </si>
+  <si>
+    <t>LR J/P</t>
+  </si>
+  <si>
+    <t>0: 0.51
+1: 0.69</t>
+  </si>
+  <si>
+    <t>0: 0.57
+1: 0.63</t>
+  </si>
+  <si>
+    <t>0: 0.54
+1: 0.66</t>
+  </si>
+  <si>
+    <t>[[197 147]
+ [192 332]]</t>
+  </si>
+  <si>
+    <t>XGB E/I</t>
+  </si>
+  <si>
     <t>0: 0.37
 1: 0.89</t>
   </si>
   <si>
+    <t>0: 0.43
+1: 0.86</t>
+  </si>
+  <si>
+    <t>[[74 126]
+ [72 596]]</t>
+  </si>
+  <si>
+    <t>XGB S/N</t>
+  </si>
+  <si>
     <t>0: 0.42
 1: 0.88</t>
   </si>
@@ -544,6 +422,120 @@
 1: 0.92</t>
   </si>
   <si>
+    <t>[[27 93]
+ [38 710]]</t>
+  </si>
+  <si>
+    <t>XGB T/F</t>
+  </si>
+  <si>
+    <t>0: 0.75
+1: 0.79</t>
+  </si>
+  <si>
+    <t>[[298 100]
+ [98 372]]</t>
+  </si>
+  <si>
+    <t>XGB J/P</t>
+  </si>
+  <si>
+    <t>0: 0.41
+1: 0.73</t>
+  </si>
+  <si>
+    <t>[[110 234]
+ [87 437]]</t>
+  </si>
+  <si>
+    <t>LSVC E/I</t>
+  </si>
+  <si>
+    <t>LSVC S/N</t>
+  </si>
+  <si>
+    <t>0: 0.26
+1: 0.92</t>
+  </si>
+  <si>
+    <t>0: 0.58
+1: 0.74</t>
+  </si>
+  <si>
+    <t>0: 0.36
+1: 0.82</t>
+  </si>
+  <si>
+    <t>[[70 50]
+ [198 550]]</t>
+  </si>
+  <si>
+    <t>LSVC T/F</t>
+  </si>
+  <si>
+    <t>0: 0.70
+1: 0.83</t>
+  </si>
+  <si>
+    <t>0: 0.83
+1: 0.69</t>
+  </si>
+  <si>
+    <t>0: 0.76
+1: 0.76</t>
+  </si>
+  <si>
+    <t>[[331 67]
+ [144 326]]</t>
+  </si>
+  <si>
+    <t>LSVC J/P</t>
+  </si>
+  <si>
+    <t>MLPC E/I</t>
+  </si>
+  <si>
+    <t>MLPC S/N</t>
+  </si>
+  <si>
+    <t>0: 0.39
+1: 0.90</t>
+  </si>
+  <si>
+    <t>[[47 73]
+ [78 670]]</t>
+  </si>
+  <si>
+    <t>MLPC T/F</t>
+  </si>
+  <si>
+    <t>MLPC J/P</t>
+  </si>
+  <si>
+    <t>KNC E/I</t>
+  </si>
+  <si>
+    <t>KNC S/N</t>
+  </si>
+  <si>
+    <t>KNC T/F</t>
+  </si>
+  <si>
+    <t>KNC J/P</t>
+  </si>
+  <si>
+    <t>DTC E/I</t>
+  </si>
+  <si>
+    <t>DTC S/N</t>
+  </si>
+  <si>
+    <t>DTC T/F</t>
+  </si>
+  <si>
+    <t>DTC J/P</t>
+  </si>
+  <si>
     <t>0: 0.46
 1: 0.89</t>
   </si>
@@ -556,38 +548,14 @@
 1: 0.82</t>
   </si>
   <si>
-    <t>[[135 65]
- [158 510]]</t>
-  </si>
-  <si>
     <t>[[60 60]
  [159 589]]</t>
   </si>
   <si>
-    <t>0: 0.48
-1: 0.82</t>
-  </si>
-  <si>
-    <t>0: 0.36
-1: 0.88</t>
-  </si>
-  <si>
     <t>0: 0.41
 1: 0.85</t>
   </si>
   <si>
-    <t>[[72 128]
- [78 590]]</t>
-  </si>
-  <si>
-    <t>0: 0.41
-1: 0.88</t>
-  </si>
-  <si>
-    <t>[[26 94]
- [38 710]]</t>
-  </si>
-  <si>
     <t>0: 0.49
 1: 0.88</t>
   </si>
@@ -700,6 +668,34 @@
  [206 542]]</t>
   </si>
   <si>
+    <t>[[136 64]
+ [157 511]]</t>
+  </si>
+  <si>
+    <t>0: 0.49
+1: 0.82</t>
+  </si>
+  <si>
+    <t>0: 0.35
+1: 0.89</t>
+  </si>
+  <si>
+    <t>[[71 129]
+ [74 594]]</t>
+  </si>
+  <si>
+    <t>0: 0.23
+1: 0.94</t>
+  </si>
+  <si>
+    <t>0: 0.29
+1: 0.91</t>
+  </si>
+  <si>
+    <t>[[27 93]
+ [42 706]]</t>
+  </si>
+  <si>
     <t>0: 0.67
 1: 0.75</t>
   </si>
@@ -720,30 +716,6 @@
 1: 0.76</t>
   </si>
   <si>
-    <t>[[60 60]
- [179 569]]</t>
-  </si>
-  <si>
-    <t>0: 0.50
-1: 0.84</t>
-  </si>
-  <si>
-    <t>0: 0.43
-1: 0.87</t>
-  </si>
-  <si>
-    <t>0: 0.47
-1: 0.85</t>
-  </si>
-  <si>
-    <t>[[87 113]
- [87 581]]</t>
-  </si>
-  <si>
-    <t>[[27 93]
- [37 711]]</t>
-  </si>
-  <si>
     <t>0: 0.74
 1: 0.72</t>
   </si>
@@ -752,18 +724,6 @@
  [190 478]]</t>
   </si>
   <si>
-    <t>0: 0.53
-1: 0.78</t>
-  </si>
-  <si>
-    <t>0: 0.37
-1: 0.84</t>
-  </si>
-  <si>
-    <t>[[64 56]
- [163 585]]</t>
-  </si>
-  <si>
     <t>0: 0.40
 1: 0.89</t>
   </si>
@@ -780,14 +740,6 @@
  [217 451]]</t>
   </si>
   <si>
-    <t>0: 0.33
-1: 0.89</t>
-  </si>
-  <si>
-    <t>[[40 80]
- [82 666]]</t>
-  </si>
-  <si>
     <t>0: 0.26
 1: 0.83</t>
   </si>
@@ -844,6 +796,70 @@
  [233 515]]</t>
   </si>
   <si>
+    <t>0: 0.34
+1: 0.83</t>
+  </si>
+  <si>
+    <t>[[60 60]
+ [177 571]]</t>
+  </si>
+  <si>
+    <t>0: 0.53
+1: 0.83</t>
+  </si>
+  <si>
+    <t>0: 0.41
+1: 0.89</t>
+  </si>
+  <si>
+    <t>0: 0.46
+1: 0.86</t>
+  </si>
+  <si>
+    <t>[[82 118]
+ [72 596]]</t>
+  </si>
+  <si>
+    <t>0: 0.38
+1: 0.88</t>
+  </si>
+  <si>
+    <t>0: 0.20
+1: 0.95</t>
+  </si>
+  <si>
+    <t>0: 0.26
+1: 0.91</t>
+  </si>
+  <si>
+    <t>[[24 96]
+ [39 709]]</t>
+  </si>
+  <si>
+    <t>0: 0.47
+1: 0.82</t>
+  </si>
+  <si>
+    <t>0: 0.36
+1: 0.86</t>
+  </si>
+  <si>
+    <t>[[56 64]
+ [135 613]]</t>
+  </si>
+  <si>
+    <t>0: 0.31
+1: 0.89</t>
+  </si>
+  <si>
+    <t>0: 0.32
+1: 0.89</t>
+  </si>
+  <si>
+    <t>[[38 82]
+ [85 663]]</t>
+  </si>
+  <si>
     <t>0: 0.72
 1: 0.67</t>
   </si>
@@ -860,58 +876,14 @@
 1: 0.91</t>
   </si>
   <si>
-    <t>0: 0.54
-1: 0.73</t>
-  </si>
-  <si>
     <t>0: 0.33
 1: 0.81</t>
   </si>
   <si>
-    <t>[[65 55]
- [205 543]]</t>
-  </si>
-  <si>
-    <t>0: 0.42
-1: 0.85</t>
-  </si>
-  <si>
-    <t>0: 0.47
-1: 0.81</t>
-  </si>
-  <si>
-    <t>[[105 95]
- [146 522]]</t>
-  </si>
-  <si>
-    <t>0: 0.48
-1: 0.87</t>
-  </si>
-  <si>
-    <t>0: 0.12
-1: 0.98</t>
-  </si>
-  <si>
-    <t>0: 0.20
-1: 0.92</t>
-  </si>
-  <si>
-    <t>[[15 105]
- [16 732]]</t>
-  </si>
-  <si>
-    <t>0: 0.46
-1: 0.88</t>
-  </si>
-  <si>
     <t>0: 0.66
 1: 0.77</t>
   </si>
   <si>
-    <t>0: 0.54
-1: 0.82</t>
-  </si>
-  <si>
     <t>[[131 69]
  [153 515]]</t>
   </si>
@@ -1020,6 +992,42 @@
  [132 616]]</t>
   </si>
   <si>
+    <t>0: 0.54
+1: 0.72</t>
+  </si>
+  <si>
+    <t>[[65 55]
+ [206 542]]</t>
+  </si>
+  <si>
+    <t>0: 0.43
+1: 0.85</t>
+  </si>
+  <si>
+    <t>0: 0.52
+1: 0.80</t>
+  </si>
+  <si>
+    <t>[[103 97]
+ [136 532]]</t>
+  </si>
+  <si>
+    <t>0: 0.47
+1: 0.88</t>
+  </si>
+  <si>
+    <t>0: 0.15
+1: 0.97</t>
+  </si>
+  <si>
+    <t>0: 0.23
+1: 0.92</t>
+  </si>
+  <si>
+    <t>[[18 102]
+ [20 728]]</t>
+  </si>
+  <si>
     <t>0: 0.74
 1: 0.63</t>
   </si>
@@ -1028,10 +1036,6 @@
 1: 0.74</t>
   </si>
   <si>
-    <t>[[149 51]
- [245 423]]</t>
-  </si>
-  <si>
     <t>0: 0.23
 1: 0.91</t>
   </si>
@@ -1052,38 +1056,10 @@
 1: 0.87</t>
   </si>
   <si>
-    <t>0: 0.68
-1: 0.66</t>
-  </si>
-  <si>
     <t>0: 0.48
 1: 0.75</t>
   </si>
   <si>
-    <t>[[136 64]
- [230 438]]</t>
-  </si>
-  <si>
-    <t>0: 0.34
-1: 0.87</t>
-  </si>
-  <si>
-    <t>0: 0.12
-1: 0.96</t>
-  </si>
-  <si>
-    <t>0: 0.18
-1: 0.91</t>
-  </si>
-  <si>
-    <t>[[15 105]
- [29 719]]</t>
-  </si>
-  <si>
-    <t>0: 0.35
-1: 0.89</t>
-  </si>
-  <si>
     <t>0: 0.77
 1: 0.57</t>
   </si>
@@ -1096,10 +1072,6 @@
  [287 381]]</t>
   </si>
   <si>
-    <t>0: 0.29
-1: 0.91</t>
-  </si>
-  <si>
     <t>0: 0.54
 1: 0.79</t>
   </si>
@@ -1198,6 +1170,30 @@
   <si>
     <t>[[40 80]
  [158 590]]</t>
+  </si>
+  <si>
+    <t>[[149 51]
+ [246 422]]</t>
+  </si>
+  <si>
+    <t>0: 0.69
+1: 0.65</t>
+  </si>
+  <si>
+    <t>[[137 63]
+ [232 436]]</t>
+  </si>
+  <si>
+    <t>0: 0.16
+1: 0.97</t>
+  </si>
+  <si>
+    <t>0: 0.24
+1: 0.92</t>
+  </si>
+  <si>
+    <t>[[19 101]
+ [22 726]]</t>
   </si>
 </sst>
 </file>
@@ -1761,613 +1757,613 @@
     </row>
     <row r="2" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>9</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>11</v>
       </c>
       <c r="F2" s="6">
         <v>0.74</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>13</v>
+        <v>86</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>15</v>
+        <v>87</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F3" s="6">
         <v>0.72</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>18</v>
+        <v>88</v>
       </c>
       <c r="H3" s="1"/>
       <c r="J3" s="14" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F4" s="6">
         <v>0.76</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F5" s="6">
         <v>0.61</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="H5" s="1"/>
     </row>
     <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>33</v>
+        <v>96</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>35</v>
+        <v>97</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>36</v>
+        <v>98</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F7" s="8">
         <v>0.77</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="H7" s="1"/>
     </row>
     <row r="8" spans="1:11" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>39</v>
+        <v>101</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>40</v>
+        <v>102</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>41</v>
+        <v>103</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F8" s="8">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>42</v>
+        <v>104</v>
       </c>
       <c r="H8" s="1"/>
       <c r="J8" s="15" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>44</v>
+        <v>105</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>45</v>
+        <v>106</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F9" s="8">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>47</v>
+        <v>107</v>
       </c>
       <c r="H9" s="1"/>
     </row>
     <row r="10" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>51</v>
+        <v>109</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F10" s="8">
         <v>0.63</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>52</v>
+        <v>110</v>
       </c>
       <c r="H10" s="1"/>
     </row>
     <row r="12" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
-        <v>53</v>
+        <v>111</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F12" s="10">
         <v>0.73</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="H12" s="1"/>
     </row>
     <row r="13" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
-        <v>58</v>
+        <v>112</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>59</v>
+        <v>113</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F13" s="10">
-        <v>0.74</v>
+        <v>0.71</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>62</v>
+        <v>116</v>
       </c>
       <c r="H13" s="1"/>
       <c r="J13" s="16" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>65</v>
+        <v>118</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>66</v>
+        <v>119</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>67</v>
+        <v>120</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F14" s="10">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>68</v>
+        <v>121</v>
       </c>
       <c r="H14" s="1"/>
     </row>
     <row r="15" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
-        <v>69</v>
+        <v>122</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F15" s="10">
         <v>0.56000000000000005</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="H15" s="1"/>
     </row>
     <row r="17" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>77</v>
+        <v>37</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F17" s="12">
         <v>0.7</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="H17" s="1"/>
     </row>
     <row r="18" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>79</v>
+        <v>124</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>81</v>
+        <v>125</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F18" s="12">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>83</v>
+        <v>126</v>
       </c>
       <c r="H18" s="1"/>
       <c r="J18" s="17" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>85</v>
+        <v>127</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F19" s="12">
         <v>0.78</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="H19" s="1"/>
     </row>
     <row r="20" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>90</v>
+        <v>128</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F20" s="12">
         <v>0.66</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="H20" s="1"/>
     </row>
     <row r="22" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="24" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>96</v>
+        <v>50</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>97</v>
+        <v>51</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>98</v>
+        <v>52</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F22" s="25">
         <v>0.48</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>99</v>
+        <v>53</v>
       </c>
       <c r="H22" s="1"/>
     </row>
     <row r="23" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="24" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>101</v>
+        <v>54</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>102</v>
+        <v>55</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>103</v>
+        <v>56</v>
       </c>
       <c r="E23" s="25" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F23" s="25">
         <v>0.47</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>104</v>
+        <v>57</v>
       </c>
       <c r="H23" s="1"/>
       <c r="J23" s="24" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K23" s="26" t="s">
-        <v>105</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="24" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="E24" s="25" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F24" s="25">
         <v>0.61</v>
       </c>
       <c r="G24" s="26" t="s">
-        <v>108</v>
+        <v>60</v>
       </c>
       <c r="H24" s="1"/>
     </row>
     <row r="25" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>110</v>
+        <v>61</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>111</v>
+        <v>62</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>112</v>
+        <v>63</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F25" s="25">
         <v>0.56000000000000005</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>113</v>
+        <v>64</v>
       </c>
       <c r="H25" s="1"/>
     </row>
     <row r="27" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="27" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="B27" s="28" t="s">
-        <v>115</v>
+        <v>65</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>116</v>
+        <v>66</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>117</v>
+        <v>67</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F27" s="28">
         <v>0.6</v>
       </c>
       <c r="G27" s="29" t="s">
-        <v>118</v>
+        <v>68</v>
       </c>
       <c r="H27" s="1"/>
     </row>
     <row r="28" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="27" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="B28" s="28" t="s">
-        <v>120</v>
+        <v>69</v>
       </c>
       <c r="C28" s="28" t="s">
-        <v>121</v>
+        <v>70</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>122</v>
+        <v>71</v>
       </c>
       <c r="E28" s="28" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F28" s="28">
         <v>0.65</v>
       </c>
       <c r="G28" s="29" t="s">
-        <v>123</v>
+        <v>72</v>
       </c>
       <c r="H28" s="1"/>
       <c r="J28" s="27" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K28" s="29" t="s">
-        <v>124</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="27" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="B29" s="28" t="s">
-        <v>126</v>
+        <v>74</v>
       </c>
       <c r="C29" s="28" t="s">
-        <v>127</v>
+        <v>75</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>128</v>
+        <v>76</v>
       </c>
       <c r="E29" s="28" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F29" s="28">
         <v>0.63</v>
       </c>
       <c r="G29" s="29" t="s">
-        <v>129</v>
+        <v>77</v>
       </c>
       <c r="H29" s="1"/>
     </row>
     <row r="30" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="27" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B30" s="28" t="s">
-        <v>131</v>
+        <v>78</v>
       </c>
       <c r="C30" s="28" t="s">
-        <v>132</v>
+        <v>79</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>133</v>
+        <v>80</v>
       </c>
       <c r="E30" s="28" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F30" s="28">
         <v>0.54</v>
       </c>
       <c r="G30" s="29" t="s">
-        <v>134</v>
+        <v>81</v>
       </c>
       <c r="H30" s="1"/>
     </row>
@@ -2419,25 +2415,25 @@
     </row>
     <row r="2" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>141</v>
-      </c>
       <c r="E2" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F2" s="6">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>142</v>
+        <v>170</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -2446,56 +2442,56 @@
     </row>
     <row r="3" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>13</v>
+        <v>86</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>77</v>
+        <v>37</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F3" s="6">
         <v>0.75</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="7" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F4" s="6">
         <v>0.76</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -2504,25 +2500,25 @@
     </row>
     <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F5" s="6">
         <v>0.61</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -2544,25 +2540,25 @@
     </row>
     <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>33</v>
+        <v>96</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>144</v>
+        <v>171</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>145</v>
+        <v>172</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F7" s="8">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>147</v>
+        <v>173</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -2571,56 +2567,56 @@
     </row>
     <row r="8" spans="1:11" ht="95.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>148</v>
+        <v>21</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>40</v>
+        <v>174</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>41</v>
+        <v>175</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F8" s="8">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="9" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>44</v>
+        <v>105</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>45</v>
+        <v>106</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F9" s="8">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>47</v>
+        <v>107</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -2629,25 +2625,25 @@
     </row>
     <row r="10" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>51</v>
+        <v>109</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F10" s="8">
         <v>0.63</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>52</v>
+        <v>110</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -2669,25 +2665,25 @@
     </row>
     <row r="12" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>53</v>
+        <v>111</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F12" s="10">
         <v>0.76</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -2696,56 +2692,56 @@
     </row>
     <row r="13" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>58</v>
+        <v>112</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F13" s="10">
         <v>0.77</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="11" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>65</v>
+        <v>118</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>66</v>
+        <v>119</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>67</v>
+        <v>120</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F14" s="10">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>68</v>
+        <v>121</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
@@ -2754,25 +2750,25 @@
     </row>
     <row r="15" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>69</v>
+        <v>122</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F15" s="10">
         <v>0.56000000000000005</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
@@ -2794,25 +2790,25 @@
     </row>
     <row r="17" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>77</v>
+        <v>37</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F17" s="12">
         <v>0.72</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
@@ -2821,56 +2817,56 @@
     </row>
     <row r="18" spans="1:11" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>79</v>
+        <v>124</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>135</v>
+        <v>97</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F18" s="12">
         <v>0.82</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="13" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>85</v>
+        <v>127</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F19" s="12">
         <v>0.78</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
@@ -2879,25 +2875,25 @@
     </row>
     <row r="20" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>90</v>
+        <v>128</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F20" s="12">
         <v>0.66</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -2919,25 +2915,25 @@
     </row>
     <row r="22" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F22" s="25">
         <v>0.48</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
@@ -2946,56 +2942,56 @@
     </row>
     <row r="23" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>101</v>
+        <v>54</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="E23" s="25" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F23" s="25">
         <v>0.49</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="26" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K23" s="26" t="s">
-        <v>105</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="26" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="E24" s="25" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F24" s="25">
         <v>0.61</v>
       </c>
       <c r="G24" s="26" t="s">
-        <v>108</v>
+        <v>60</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
@@ -3004,25 +3000,25 @@
     </row>
     <row r="25" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="26" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>110</v>
+        <v>61</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>111</v>
+        <v>62</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>112</v>
+        <v>63</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F25" s="25">
         <v>0.56000000000000005</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>113</v>
+        <v>64</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
@@ -3044,25 +3040,25 @@
     </row>
     <row r="27" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="29" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="B27" s="28" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F27" s="28">
         <v>0.62</v>
       </c>
       <c r="G27" s="29" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
@@ -3071,56 +3067,56 @@
     </row>
     <row r="28" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="29" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="B28" s="28" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="C28" s="28" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="E28" s="28" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F28" s="28">
         <v>0.68</v>
       </c>
       <c r="G28" s="29" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="29" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K28" s="29" t="s">
-        <v>124</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="29" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="B29" s="28" t="s">
-        <v>126</v>
+        <v>74</v>
       </c>
       <c r="C29" s="28" t="s">
-        <v>127</v>
+        <v>75</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>128</v>
+        <v>76</v>
       </c>
       <c r="E29" s="28" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F29" s="28">
         <v>0.63</v>
       </c>
       <c r="G29" s="29" t="s">
-        <v>129</v>
+        <v>77</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
@@ -3129,25 +3125,25 @@
     </row>
     <row r="30" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="29" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B30" s="28" t="s">
-        <v>131</v>
+        <v>78</v>
       </c>
       <c r="C30" s="28" t="s">
-        <v>132</v>
+        <v>79</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>133</v>
+        <v>80</v>
       </c>
       <c r="E30" s="28" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F30" s="28">
         <v>0.54</v>
       </c>
       <c r="G30" s="29" t="s">
-        <v>134</v>
+        <v>81</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
@@ -3199,25 +3195,25 @@
     </row>
     <row r="2" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>8</v>
-      </c>
       <c r="C2" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>179</v>
-      </c>
       <c r="E2" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F2" s="6">
         <v>0.73</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -3226,56 +3222,56 @@
     </row>
     <row r="3" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>13</v>
+        <v>86</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>182</v>
-      </c>
       <c r="D3" s="6" t="s">
-        <v>50</v>
+        <v>202</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F3" s="6">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="7" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F4" s="6">
         <v>0.76</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -3284,25 +3280,25 @@
     </row>
     <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F5" s="6">
         <v>0.61</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -3324,25 +3320,25 @@
     </row>
     <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>33</v>
+        <v>96</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>186</v>
+        <v>206</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F7" s="8">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -3351,56 +3347,56 @@
     </row>
     <row r="8" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>136</v>
+        <v>208</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>137</v>
+        <v>209</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>138</v>
+        <v>210</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F8" s="8">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>188</v>
+        <v>211</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="9" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>44</v>
+        <v>105</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>45</v>
+        <v>106</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F9" s="8">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>47</v>
+        <v>107</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -3409,25 +3405,25 @@
     </row>
     <row r="10" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>51</v>
+        <v>109</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F10" s="8">
         <v>0.63</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>52</v>
+        <v>110</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -3449,25 +3445,25 @@
     </row>
     <row r="12" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>53</v>
+        <v>111</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F12" s="10">
         <v>0.72</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -3476,56 +3472,56 @@
     </row>
     <row r="13" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>58</v>
+        <v>112</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>41</v>
+        <v>175</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F13" s="10">
-        <v>0.75</v>
+        <v>0.77</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>193</v>
+        <v>214</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="11" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>65</v>
+        <v>118</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>66</v>
+        <v>119</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>67</v>
+        <v>120</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F14" s="10">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>68</v>
+        <v>121</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
@@ -3534,25 +3530,25 @@
     </row>
     <row r="15" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>69</v>
+        <v>122</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F15" s="10">
         <v>0.56000000000000005</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
@@ -3574,25 +3570,25 @@
     </row>
     <row r="17" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F17" s="12">
         <v>0.68</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
@@ -3601,56 +3597,56 @@
     </row>
     <row r="18" spans="1:11" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>79</v>
+        <v>124</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>198</v>
+        <v>216</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F18" s="12">
         <v>0.81</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>199</v>
+        <v>217</v>
       </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="13" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>85</v>
+        <v>127</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F19" s="12">
         <v>0.78</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
@@ -3659,25 +3655,25 @@
     </row>
     <row r="20" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>90</v>
+        <v>128</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F20" s="12">
         <v>0.66</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -3699,25 +3695,25 @@
     </row>
     <row r="22" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F22" s="25">
         <v>0.45</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
@@ -3726,56 +3722,56 @@
     </row>
     <row r="23" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>103</v>
+        <v>56</v>
       </c>
       <c r="E23" s="25" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F23" s="25">
         <v>0.47</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="26" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K23" s="26" t="s">
-        <v>105</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="26" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="E24" s="25" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F24" s="25">
         <v>0.61</v>
       </c>
       <c r="G24" s="26" t="s">
-        <v>108</v>
+        <v>60</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
@@ -3784,25 +3780,25 @@
     </row>
     <row r="25" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="26" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>110</v>
+        <v>61</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>111</v>
+        <v>62</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>112</v>
+        <v>63</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F25" s="25">
         <v>0.56000000000000005</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>113</v>
+        <v>64</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
@@ -3824,25 +3820,25 @@
     </row>
     <row r="27" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="29" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="B27" s="28" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F27" s="28">
         <v>0.63</v>
       </c>
       <c r="G27" s="29" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
@@ -3851,56 +3847,56 @@
     </row>
     <row r="28" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="29" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="B28" s="28" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="C28" s="28" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="E28" s="28" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F28" s="28">
         <v>0.63</v>
       </c>
       <c r="G28" s="29" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="29" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K28" s="29" t="s">
-        <v>124</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="29" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="B29" s="28" t="s">
-        <v>126</v>
+        <v>74</v>
       </c>
       <c r="C29" s="28" t="s">
-        <v>127</v>
+        <v>75</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>128</v>
+        <v>76</v>
       </c>
       <c r="E29" s="28" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F29" s="28">
         <v>0.63</v>
       </c>
       <c r="G29" s="29" t="s">
-        <v>129</v>
+        <v>77</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
@@ -3909,25 +3905,25 @@
     </row>
     <row r="30" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="29" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B30" s="28" t="s">
-        <v>131</v>
+        <v>78</v>
       </c>
       <c r="C30" s="28" t="s">
-        <v>132</v>
+        <v>79</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>133</v>
+        <v>80</v>
       </c>
       <c r="E30" s="28" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F30" s="28">
         <v>0.54</v>
       </c>
       <c r="G30" s="29" t="s">
-        <v>134</v>
+        <v>81</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
@@ -3950,8 +3946,8 @@
     <col min="8" max="9" width="9.140625" style="1" customWidth="1"/>
     <col min="10" max="10" width="13.42578125" style="1" customWidth="1"/>
     <col min="11" max="11" width="45.85546875" style="1" customWidth="1"/>
-    <col min="12" max="14" width="9.140625" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="1"/>
+    <col min="12" max="15" width="9.140625" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -3979,104 +3975,104 @@
     </row>
     <row r="2" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F2" s="6">
         <v>0.69</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
     </row>
     <row r="3" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>13</v>
+        <v>86</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>218</v>
+        <v>251</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F3" s="6">
         <v>0.7</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>220</v>
+        <v>252</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F4" s="6">
         <v>0.76</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
     <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F5" s="6">
         <v>0.61</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
@@ -4089,104 +4085,104 @@
     </row>
     <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>33</v>
+        <v>96</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>221</v>
+        <v>253</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>191</v>
+        <v>254</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F7" s="8">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>223</v>
+        <v>255</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
     <row r="8" spans="1:11" ht="141" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>224</v>
+        <v>256</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>225</v>
+        <v>257</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>226</v>
+        <v>258</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F8" s="8">
         <v>0.86</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>227</v>
+        <v>259</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>44</v>
+        <v>105</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>45</v>
+        <v>106</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F9" s="8">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>47</v>
+        <v>107</v>
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
     <row r="10" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>51</v>
+        <v>109</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F10" s="8">
         <v>0.63</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>52</v>
+        <v>110</v>
       </c>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
@@ -4199,104 +4195,104 @@
     </row>
     <row r="12" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>53</v>
+        <v>111</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>228</v>
+        <v>83</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>230</v>
+        <v>84</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F12" s="10">
         <v>0.74</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
     </row>
     <row r="13" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>58</v>
+        <v>112</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F13" s="10">
         <v>0.51</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>65</v>
+        <v>118</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>66</v>
+        <v>119</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>67</v>
+        <v>120</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F14" s="10">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>68</v>
+        <v>121</v>
       </c>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
     </row>
     <row r="15" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>69</v>
+        <v>122</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F15" s="10">
         <v>0.56000000000000005</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
@@ -4309,104 +4305,104 @@
     </row>
     <row r="17" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F17" s="12">
         <v>0.66</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
     </row>
     <row r="18" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>79</v>
+        <v>124</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F18" s="12">
         <v>0.84</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>85</v>
+        <v>127</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F19" s="12">
         <v>0.78</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
     </row>
     <row r="20" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>90</v>
+        <v>128</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F20" s="12">
         <v>0.66</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
@@ -4419,104 +4415,104 @@
     </row>
     <row r="22" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>115</v>
+        <v>65</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F22" s="25">
         <v>0.61</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
     </row>
     <row r="23" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>120</v>
+        <v>69</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="E23" s="25" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F23" s="25">
         <v>0.75</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="J23" s="26" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K23" s="26" t="s">
-        <v>105</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="26" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="E24" s="25" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F24" s="25">
         <v>0.61</v>
       </c>
       <c r="G24" s="26" t="s">
-        <v>108</v>
+        <v>60</v>
       </c>
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
     </row>
     <row r="25" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="26" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>110</v>
+        <v>61</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>111</v>
+        <v>62</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>112</v>
+        <v>63</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F25" s="25">
         <v>0.56000000000000005</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>113</v>
+        <v>64</v>
       </c>
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
@@ -4529,104 +4525,104 @@
     </row>
     <row r="27" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="29" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="B27" s="28" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F27" s="28">
         <v>0.59</v>
       </c>
       <c r="G27" s="29" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
     </row>
     <row r="28" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="29" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="B28" s="28" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="C28" s="28" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="E28" s="28" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F28" s="28">
         <v>0.75</v>
       </c>
       <c r="G28" s="29" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="J28" s="29" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K28" s="29" t="s">
-        <v>124</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="29" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="B29" s="28" t="s">
-        <v>126</v>
+        <v>74</v>
       </c>
       <c r="C29" s="28" t="s">
-        <v>127</v>
+        <v>75</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>128</v>
+        <v>76</v>
       </c>
       <c r="E29" s="28" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F29" s="28">
         <v>0.63</v>
       </c>
       <c r="G29" s="29" t="s">
-        <v>129</v>
+        <v>77</v>
       </c>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
     </row>
     <row r="30" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="29" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B30" s="28" t="s">
-        <v>131</v>
+        <v>78</v>
       </c>
       <c r="C30" s="28" t="s">
-        <v>132</v>
+        <v>79</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>133</v>
+        <v>80</v>
       </c>
       <c r="E30" s="28" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F30" s="28">
         <v>0.54</v>
       </c>
       <c r="G30" s="29" t="s">
-        <v>134</v>
+        <v>81</v>
       </c>
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
@@ -4673,25 +4669,25 @@
     </row>
     <row r="2" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F2" s="6">
         <v>0.66</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>260</v>
+        <v>296</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -4700,56 +4696,56 @@
     </row>
     <row r="3" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>13</v>
+        <v>86</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F3" s="6">
         <v>0.69</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="7" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F4" s="6">
         <v>0.76</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -4758,25 +4754,25 @@
     </row>
     <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F5" s="6">
         <v>0.61</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -4798,25 +4794,25 @@
     </row>
     <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>33</v>
+        <v>96</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>267</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F7" s="8">
         <v>0.66</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>268</v>
+        <v>298</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -4825,56 +4821,56 @@
     </row>
     <row r="8" spans="1:11" ht="120" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>269</v>
+        <v>83</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>270</v>
+        <v>299</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>271</v>
+        <v>300</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F8" s="8">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="9" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>44</v>
+        <v>105</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>45</v>
+        <v>106</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F9" s="8">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>47</v>
+        <v>107</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -4883,25 +4879,25 @@
     </row>
     <row r="10" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>51</v>
+        <v>109</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F10" s="8">
         <v>0.63</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>52</v>
+        <v>110</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -4923,25 +4919,25 @@
     </row>
     <row r="12" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>53</v>
+        <v>111</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>273</v>
+        <v>172</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F12" s="10">
         <v>0.62</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -4950,56 +4946,56 @@
     </row>
     <row r="13" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>58</v>
+        <v>112</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>277</v>
+        <v>175</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F13" s="10">
         <v>0.75</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="11" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>65</v>
+        <v>118</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>66</v>
+        <v>119</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>67</v>
+        <v>120</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F14" s="10">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>68</v>
+        <v>121</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
@@ -5008,25 +5004,25 @@
     </row>
     <row r="15" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>69</v>
+        <v>122</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F15" s="10">
         <v>0.56000000000000005</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
@@ -5048,25 +5044,25 @@
     </row>
     <row r="17" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F17" s="12">
         <v>0.63</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
@@ -5075,56 +5071,56 @@
     </row>
     <row r="18" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>79</v>
+        <v>124</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F18" s="12">
         <v>0.85</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="13" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>85</v>
+        <v>127</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F19" s="12">
         <v>0.78</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
@@ -5133,25 +5129,25 @@
     </row>
     <row r="20" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>90</v>
+        <v>128</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F20" s="12">
         <v>0.66</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -5173,25 +5169,25 @@
     </row>
     <row r="22" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F22" s="25">
         <v>0.56999999999999995</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
@@ -5200,56 +5196,56 @@
     </row>
     <row r="23" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="E23" s="25" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F23" s="25">
         <v>0.74</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="26" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K23" s="26" t="s">
-        <v>105</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="26" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="E24" s="25" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F24" s="25">
         <v>0.61</v>
       </c>
       <c r="G24" s="26" t="s">
-        <v>108</v>
+        <v>60</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
@@ -5258,25 +5254,25 @@
     </row>
     <row r="25" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="26" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>110</v>
+        <v>61</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>111</v>
+        <v>62</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>112</v>
+        <v>63</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F25" s="25">
         <v>0.56000000000000005</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>113</v>
+        <v>64</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
@@ -5298,25 +5294,25 @@
     </row>
     <row r="27" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="29" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="B27" s="28" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F27" s="28">
         <v>0.56999999999999995</v>
       </c>
       <c r="G27" s="29" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
@@ -5325,56 +5321,56 @@
     </row>
     <row r="28" spans="1:11" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="29" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="B28" s="28" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="C28" s="28" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="E28" s="28" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F28" s="28">
         <v>0.73</v>
       </c>
       <c r="G28" s="29" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="29" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K28" s="29" t="s">
-        <v>124</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="29" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="B29" s="28" t="s">
-        <v>126</v>
+        <v>74</v>
       </c>
       <c r="C29" s="28" t="s">
-        <v>127</v>
+        <v>75</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>128</v>
+        <v>76</v>
       </c>
       <c r="E29" s="28" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F29" s="28">
         <v>0.63</v>
       </c>
       <c r="G29" s="29" t="s">
-        <v>129</v>
+        <v>77</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
@@ -5383,25 +5379,25 @@
     </row>
     <row r="30" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="29" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B30" s="28" t="s">
-        <v>131</v>
+        <v>78</v>
       </c>
       <c r="C30" s="28" t="s">
-        <v>132</v>
+        <v>79</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>133</v>
+        <v>80</v>
       </c>
       <c r="E30" s="28" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F30" s="28">
         <v>0.54</v>
       </c>
       <c r="G30" s="29" t="s">
-        <v>134</v>
+        <v>81</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>

</xml_diff>